<commit_message>
Exclude graded and variation listings from price estimates
</commit_message>
<xml_diff>
--- a/reports/inventory/cs5ac_radiant_eevee_listing_price_by_seller_location.xlsx
+++ b/reports/inventory/cs5ac_radiant_eevee_listing_price_by_seller_location.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="US Sellers" sheetId="1" r:id="Rdd10497102b044e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="International" sheetId="2" r:id="R97ec9a65808442f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aggregate" sheetId="3" r:id="Rb20c50d10189468b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="US Sellers" sheetId="1" r:id="R2cd255cee41c40bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="International" sheetId="2" r:id="Rbad7c0115a7144b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aggregate" sheetId="3" r:id="R9c8d47b51ce54007"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -440,31 +440,31 @@
         <x:v>us</x:v>
       </x:c>
       <x:c r="M2" s="6" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N2" s="6" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O2" s="6" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="P2" s="6" t="n">
-        <x:v>6448.25</x:v>
+        <x:v>3598</x:v>
       </x:c>
       <x:c r="Q2" s="6" t="str">
-        <x:v>$64.48</x:v>
+        <x:v>$35.98</x:v>
       </x:c>
       <x:c r="R2" s="6" t="n">
-        <x:v>9298.5</x:v>
+        <x:v>3598</x:v>
       </x:c>
       <x:c r="S2" s="6" t="str">
-        <x:v>$92.98</x:v>
+        <x:v>$35.98</x:v>
       </x:c>
       <x:c r="T2" s="6" t="n">
-        <x:v>9298.5</x:v>
+        <x:v>3598</x:v>
       </x:c>
       <x:c r="U2" s="6" t="str">
-        <x:v>$92.98</x:v>
+        <x:v>$35.98</x:v>
       </x:c>
       <x:c r="V2" s="6" t="n">
         <x:v>3598</x:v>
@@ -473,16 +473,16 @@
         <x:v>$35.98</x:v>
       </x:c>
       <x:c r="X2" s="6" t="n">
-        <x:v>14999</x:v>
+        <x:v>3598</x:v>
       </x:c>
       <x:c r="Y2" s="6" t="str">
-        <x:v>$149.99</x:v>
+        <x:v>$35.98</x:v>
       </x:c>
       <x:c r="Z2" s="6" t="n">
-        <x:v>8061.724412307828</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="AA2" s="6" t="str">
-        <x:v>$80.62</x:v>
+        <x:v>$0.00</x:v>
       </x:c>
       <x:c r="AB2" s="6" t="n">
         <x:v>100</x:v>
@@ -491,46 +491,46 @@
         <x:v>$1.00</x:v>
       </x:c>
       <x:c r="AD2" s="6" t="n">
-        <x:v>6325</x:v>
+        <x:v>3475</x:v>
       </x:c>
       <x:c r="AE2" s="6" t="str">
-        <x:v>$63.25</x:v>
+        <x:v>$34.75</x:v>
       </x:c>
       <x:c r="AF2" s="6" t="n">
-        <x:v>6325</x:v>
+        <x:v>3475</x:v>
       </x:c>
       <x:c r="AG2" s="6" t="str">
-        <x:v>$63.25</x:v>
+        <x:v>$34.75</x:v>
       </x:c>
       <x:c r="AH2" s="6" t="n">
-        <x:v>838</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="AI2" s="6" t="str">
-        <x:v>$8.38</x:v>
+        <x:v>$4.60</x:v>
       </x:c>
       <x:c r="AJ2" s="6" t="n">
-        <x:v>5487</x:v>
+        <x:v>3015</x:v>
       </x:c>
       <x:c r="AK2" s="6" t="str">
-        <x:v>$54.87</x:v>
+        <x:v>$30.15</x:v>
       </x:c>
       <x:c r="AL2" s="6" t="n">
-        <x:v>6325</x:v>
+        <x:v>3475</x:v>
       </x:c>
       <x:c r="AM2" s="6" t="str">
-        <x:v>$63.25</x:v>
+        <x:v>$34.75</x:v>
       </x:c>
       <x:c r="AN2" s="6" t="n">
-        <x:v>838</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="AO2" s="6" t="str">
-        <x:v>$8.38</x:v>
+        <x:v>$4.60</x:v>
       </x:c>
       <x:c r="AP2" s="6" t="n">
-        <x:v>5487</x:v>
+        <x:v>3015</x:v>
       </x:c>
       <x:c r="AQ2" s="6" t="str">
-        <x:v>$54.87</x:v>
+        <x:v>$30.15</x:v>
       </x:c>
       <x:c r="AR2" s="6" t="str">
         <x:v>recalculated_from_raw</x:v>
@@ -761,31 +761,31 @@
         <x:v>international</x:v>
       </x:c>
       <x:c r="M2" s="6" t="n">
-        <x:v>83</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="N2" s="6" t="n">
-        <x:v>83</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="O2" s="6" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="P2" s="6" t="n">
-        <x:v>3201</x:v>
+        <x:v>3167</x:v>
       </x:c>
       <x:c r="Q2" s="6" t="str">
-        <x:v>$32.01</x:v>
+        <x:v>$31.67</x:v>
       </x:c>
       <x:c r="R2" s="6" t="n">
-        <x:v>17566.433734939757</x:v>
+        <x:v>13630.686956521738</x:v>
       </x:c>
       <x:c r="S2" s="6" t="str">
-        <x:v>$175.66</x:v>
+        <x:v>$136.31</x:v>
       </x:c>
       <x:c r="T2" s="6" t="n">
-        <x:v>3687</x:v>
+        <x:v>3688</x:v>
       </x:c>
       <x:c r="U2" s="6" t="str">
-        <x:v>$36.87</x:v>
+        <x:v>$36.88</x:v>
       </x:c>
       <x:c r="V2" s="6" t="n">
         <x:v>2203</x:v>
@@ -800,10 +800,10 @@
         <x:v>$3,255.80</x:v>
       </x:c>
       <x:c r="Z2" s="6" t="n">
-        <x:v>55048.004500549396</x:v>
+        <x:v>47113.413076407036</x:v>
       </x:c>
       <x:c r="AA2" s="6" t="str">
-        <x:v>$550.48</x:v>
+        <x:v>$471.13</x:v>
       </x:c>
       <x:c r="AB2" s="6" t="n">
         <x:v>100</x:v>
@@ -812,46 +812,46 @@
         <x:v>$1.00</x:v>
       </x:c>
       <x:c r="AD2" s="6" t="n">
-        <x:v>3100</x:v>
+        <x:v>3050</x:v>
       </x:c>
       <x:c r="AE2" s="6" t="str">
-        <x:v>$31.00</x:v>
+        <x:v>$30.50</x:v>
       </x:c>
       <x:c r="AF2" s="6" t="n">
-        <x:v>3100</x:v>
+        <x:v>3050</x:v>
       </x:c>
       <x:c r="AG2" s="6" t="str">
-        <x:v>$31.00</x:v>
+        <x:v>$30.50</x:v>
       </x:c>
       <x:c r="AH2" s="6" t="n">
-        <x:v>411</x:v>
+        <x:v>404</x:v>
       </x:c>
       <x:c r="AI2" s="6" t="str">
-        <x:v>$4.11</x:v>
+        <x:v>$4.04</x:v>
       </x:c>
       <x:c r="AJ2" s="6" t="n">
-        <x:v>2689</x:v>
+        <x:v>2646</x:v>
       </x:c>
       <x:c r="AK2" s="6" t="str">
-        <x:v>$26.89</x:v>
+        <x:v>$26.46</x:v>
       </x:c>
       <x:c r="AL2" s="6" t="n">
-        <x:v>3100</x:v>
+        <x:v>3050</x:v>
       </x:c>
       <x:c r="AM2" s="6" t="str">
-        <x:v>$31.00</x:v>
+        <x:v>$30.50</x:v>
       </x:c>
       <x:c r="AN2" s="6" t="n">
-        <x:v>411</x:v>
+        <x:v>404</x:v>
       </x:c>
       <x:c r="AO2" s="6" t="str">
-        <x:v>$4.11</x:v>
+        <x:v>$4.04</x:v>
       </x:c>
       <x:c r="AP2" s="6" t="n">
-        <x:v>2689</x:v>
+        <x:v>2646</x:v>
       </x:c>
       <x:c r="AQ2" s="6" t="str">
-        <x:v>$26.89</x:v>
+        <x:v>$26.46</x:v>
       </x:c>
       <x:c r="AR2" s="6" t="str">
         <x:v>recalculated_from_raw</x:v>
@@ -1082,28 +1082,28 @@
         <x:v>aggregate</x:v>
       </x:c>
       <x:c r="M2" s="6" t="n">
-        <x:v>84</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="N2" s="6" t="n">
-        <x:v>84</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="O2" s="6" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="P2" s="6" t="n">
-        <x:v>3211</x:v>
+        <x:v>3173.5</x:v>
       </x:c>
       <x:c r="Q2" s="6" t="str">
-        <x:v>$32.11</x:v>
+        <x:v>$31.73</x:v>
       </x:c>
       <x:c r="R2" s="6" t="n">
-        <x:v>17535.869047619046</x:v>
+        <x:v>13544.198275862069</x:v>
       </x:c>
       <x:c r="S2" s="6" t="str">
-        <x:v>$175.36</x:v>
+        <x:v>$135.44</x:v>
       </x:c>
       <x:c r="T2" s="6" t="n">
-        <x:v>3687.5</x:v>
+        <x:v>3688</x:v>
       </x:c>
       <x:c r="U2" s="6" t="str">
         <x:v>$36.88</x:v>
@@ -1121,10 +1121,10 @@
         <x:v>$3,255.80</x:v>
       </x:c>
       <x:c r="Z2" s="6" t="n">
-        <x:v>54716.10220933729</x:v>
+        <x:v>46917.37306375777</x:v>
       </x:c>
       <x:c r="AA2" s="6" t="str">
-        <x:v>$547.16</x:v>
+        <x:v>$469.17</x:v>
       </x:c>
       <x:c r="AB2" s="6" t="n">
         <x:v>100</x:v>
@@ -1133,46 +1133,46 @@
         <x:v>$1.00</x:v>
       </x:c>
       <x:c r="AD2" s="6" t="n">
-        <x:v>3100</x:v>
+        <x:v>3050</x:v>
       </x:c>
       <x:c r="AE2" s="6" t="str">
-        <x:v>$31.00</x:v>
+        <x:v>$30.50</x:v>
       </x:c>
       <x:c r="AF2" s="6" t="n">
-        <x:v>3100</x:v>
+        <x:v>3050</x:v>
       </x:c>
       <x:c r="AG2" s="6" t="str">
-        <x:v>$31.00</x:v>
+        <x:v>$30.50</x:v>
       </x:c>
       <x:c r="AH2" s="6" t="n">
-        <x:v>411</x:v>
+        <x:v>404</x:v>
       </x:c>
       <x:c r="AI2" s="6" t="str">
-        <x:v>$4.11</x:v>
+        <x:v>$4.04</x:v>
       </x:c>
       <x:c r="AJ2" s="6" t="n">
-        <x:v>2689</x:v>
+        <x:v>2646</x:v>
       </x:c>
       <x:c r="AK2" s="6" t="str">
-        <x:v>$26.89</x:v>
+        <x:v>$26.46</x:v>
       </x:c>
       <x:c r="AL2" s="6" t="n">
-        <x:v>3100</x:v>
+        <x:v>3050</x:v>
       </x:c>
       <x:c r="AM2" s="6" t="str">
-        <x:v>$31.00</x:v>
+        <x:v>$30.50</x:v>
       </x:c>
       <x:c r="AN2" s="6" t="n">
-        <x:v>411</x:v>
+        <x:v>404</x:v>
       </x:c>
       <x:c r="AO2" s="6" t="str">
-        <x:v>$4.11</x:v>
+        <x:v>$4.04</x:v>
       </x:c>
       <x:c r="AP2" s="6" t="n">
-        <x:v>2689</x:v>
+        <x:v>2646</x:v>
       </x:c>
       <x:c r="AQ2" s="6" t="str">
-        <x:v>$26.89</x:v>
+        <x:v>$26.46</x:v>
       </x:c>
       <x:c r="AR2" s="6" t="str">
         <x:v>recalculated_from_raw</x:v>

</xml_diff>

<commit_message>
Refresh Radiant Eevee pricing report
</commit_message>
<xml_diff>
--- a/reports/inventory/cs5ac_radiant_eevee_listing_price_by_seller_location.xlsx
+++ b/reports/inventory/cs5ac_radiant_eevee_listing_price_by_seller_location.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="US Sellers" sheetId="1" r:id="R2cd255cee41c40bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="International" sheetId="2" r:id="Rbad7c0115a7144b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aggregate" sheetId="3" r:id="R9c8d47b51ce54007"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="US Sellers" sheetId="1" r:id="R0963633a06d24f6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="International" sheetId="2" r:id="Ra48764edbbe04d25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aggregate" sheetId="3" r:id="R29562cd22f344893"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -440,25 +440,25 @@
         <x:v>us</x:v>
       </x:c>
       <x:c r="M2" s="6" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N2" s="6" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="O2" s="6" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="P2" s="6" t="n">
-        <x:v>3598</x:v>
+        <x:v>3499</x:v>
       </x:c>
       <x:c r="Q2" s="6" t="str">
-        <x:v>$35.98</x:v>
+        <x:v>$34.99</x:v>
       </x:c>
       <x:c r="R2" s="6" t="n">
-        <x:v>3598</x:v>
+        <x:v>3999.3333333333335</x:v>
       </x:c>
       <x:c r="S2" s="6" t="str">
-        <x:v>$35.98</x:v>
+        <x:v>$39.99</x:v>
       </x:c>
       <x:c r="T2" s="6" t="n">
         <x:v>3598</x:v>
@@ -467,22 +467,22 @@
         <x:v>$35.98</x:v>
       </x:c>
       <x:c r="V2" s="6" t="n">
-        <x:v>3598</x:v>
+        <x:v>3400</x:v>
       </x:c>
       <x:c r="W2" s="6" t="str">
-        <x:v>$35.98</x:v>
+        <x:v>$34.00</x:v>
       </x:c>
       <x:c r="X2" s="6" t="n">
-        <x:v>3598</x:v>
+        <x:v>5000</x:v>
       </x:c>
       <x:c r="Y2" s="6" t="str">
-        <x:v>$35.98</x:v>
+        <x:v>$50.00</x:v>
       </x:c>
       <x:c r="Z2" s="6" t="n">
-        <x:v>0</x:v>
+        <x:v>872.2392638108728</x:v>
       </x:c>
       <x:c r="AA2" s="6" t="str">
-        <x:v>$0.00</x:v>
+        <x:v>$8.72</x:v>
       </x:c>
       <x:c r="AB2" s="6" t="n">
         <x:v>100</x:v>
@@ -491,46 +491,46 @@
         <x:v>$1.00</x:v>
       </x:c>
       <x:c r="AD2" s="6" t="n">
-        <x:v>3475</x:v>
+        <x:v>3375</x:v>
       </x:c>
       <x:c r="AE2" s="6" t="str">
-        <x:v>$34.75</x:v>
+        <x:v>$33.75</x:v>
       </x:c>
       <x:c r="AF2" s="6" t="n">
-        <x:v>3475</x:v>
+        <x:v>3375</x:v>
       </x:c>
       <x:c r="AG2" s="6" t="str">
-        <x:v>$34.75</x:v>
+        <x:v>$33.75</x:v>
       </x:c>
       <x:c r="AH2" s="6" t="n">
-        <x:v>460</x:v>
+        <x:v>447</x:v>
       </x:c>
       <x:c r="AI2" s="6" t="str">
-        <x:v>$4.60</x:v>
+        <x:v>$4.47</x:v>
       </x:c>
       <x:c r="AJ2" s="6" t="n">
-        <x:v>3015</x:v>
+        <x:v>2928</x:v>
       </x:c>
       <x:c r="AK2" s="6" t="str">
-        <x:v>$30.15</x:v>
+        <x:v>$29.28</x:v>
       </x:c>
       <x:c r="AL2" s="6" t="n">
-        <x:v>3475</x:v>
+        <x:v>3375</x:v>
       </x:c>
       <x:c r="AM2" s="6" t="str">
-        <x:v>$34.75</x:v>
+        <x:v>$33.75</x:v>
       </x:c>
       <x:c r="AN2" s="6" t="n">
-        <x:v>460</x:v>
+        <x:v>447</x:v>
       </x:c>
       <x:c r="AO2" s="6" t="str">
-        <x:v>$4.60</x:v>
+        <x:v>$4.47</x:v>
       </x:c>
       <x:c r="AP2" s="6" t="n">
-        <x:v>3015</x:v>
+        <x:v>2928</x:v>
       </x:c>
       <x:c r="AQ2" s="6" t="str">
-        <x:v>$30.15</x:v>
+        <x:v>$29.28</x:v>
       </x:c>
       <x:c r="AR2" s="6" t="str">
         <x:v>recalculated_from_raw</x:v>
@@ -1082,25 +1082,25 @@
         <x:v>aggregate</x:v>
       </x:c>
       <x:c r="M2" s="6" t="n">
-        <x:v>116</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="N2" s="6" t="n">
-        <x:v>116</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="O2" s="6" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="P2" s="6" t="n">
-        <x:v>3173.5</x:v>
+        <x:v>3180.25</x:v>
       </x:c>
       <x:c r="Q2" s="6" t="str">
-        <x:v>$31.73</x:v>
+        <x:v>$31.80</x:v>
       </x:c>
       <x:c r="R2" s="6" t="n">
-        <x:v>13544.198275862069</x:v>
+        <x:v>13385.822033898305</x:v>
       </x:c>
       <x:c r="S2" s="6" t="str">
-        <x:v>$135.44</x:v>
+        <x:v>$133.86</x:v>
       </x:c>
       <x:c r="T2" s="6" t="n">
         <x:v>3688</x:v>
@@ -1121,10 +1121,10 @@
         <x:v>$3,255.80</x:v>
       </x:c>
       <x:c r="Z2" s="6" t="n">
-        <x:v>46917.37306375777</x:v>
+        <x:v>46530.52818608176</x:v>
       </x:c>
       <x:c r="AA2" s="6" t="str">
-        <x:v>$469.17</x:v>
+        <x:v>$465.31</x:v>
       </x:c>
       <x:c r="AB2" s="6" t="n">
         <x:v>100</x:v>
@@ -1133,46 +1133,46 @@
         <x:v>$1.00</x:v>
       </x:c>
       <x:c r="AD2" s="6" t="n">
-        <x:v>3050</x:v>
+        <x:v>3075</x:v>
       </x:c>
       <x:c r="AE2" s="6" t="str">
-        <x:v>$30.50</x:v>
+        <x:v>$30.75</x:v>
       </x:c>
       <x:c r="AF2" s="6" t="n">
-        <x:v>3050</x:v>
+        <x:v>3075</x:v>
       </x:c>
       <x:c r="AG2" s="6" t="str">
-        <x:v>$30.50</x:v>
+        <x:v>$30.75</x:v>
       </x:c>
       <x:c r="AH2" s="6" t="n">
-        <x:v>404</x:v>
+        <x:v>407</x:v>
       </x:c>
       <x:c r="AI2" s="6" t="str">
-        <x:v>$4.04</x:v>
+        <x:v>$4.07</x:v>
       </x:c>
       <x:c r="AJ2" s="6" t="n">
-        <x:v>2646</x:v>
+        <x:v>2668</x:v>
       </x:c>
       <x:c r="AK2" s="6" t="str">
-        <x:v>$26.46</x:v>
+        <x:v>$26.68</x:v>
       </x:c>
       <x:c r="AL2" s="6" t="n">
-        <x:v>3050</x:v>
+        <x:v>3075</x:v>
       </x:c>
       <x:c r="AM2" s="6" t="str">
-        <x:v>$30.50</x:v>
+        <x:v>$30.75</x:v>
       </x:c>
       <x:c r="AN2" s="6" t="n">
-        <x:v>404</x:v>
+        <x:v>407</x:v>
       </x:c>
       <x:c r="AO2" s="6" t="str">
-        <x:v>$4.04</x:v>
+        <x:v>$4.07</x:v>
       </x:c>
       <x:c r="AP2" s="6" t="n">
-        <x:v>2646</x:v>
+        <x:v>2668</x:v>
       </x:c>
       <x:c r="AQ2" s="6" t="str">
-        <x:v>$26.46</x:v>
+        <x:v>$26.68</x:v>
       </x:c>
       <x:c r="AR2" s="6" t="str">
         <x:v>recalculated_from_raw</x:v>

</xml_diff>